<commit_message>
Update reports 2026-09-04 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-04.xlsx
+++ b/gex_pivot_levels_2026-09-04.xlsx
@@ -19,8 +19,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -602,12 +602,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$4.50M</t>
+          <t>-$3.94M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$9.70M</t>
+          <t>+$8.49M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -664,12 +664,12 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>-$11.05M</t>
+          <t>-$9.92M</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>+$45.97M</t>
+          <t>+$41.28M</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -697,12 +697,12 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>+$4.35M</t>
+          <t>+$3.95M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$21.62M</t>
+          <t>+$19.63M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>-$7.18M</t>
+          <t>-$6.58M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$28.19M</t>
+          <t>+$25.80M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -792,12 +792,12 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>+$70.66K</t>
+          <t>+$65.08K</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>+$33.13M</t>
+          <t>+$30.51M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -854,12 +854,12 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>+$6.36M</t>
+          <t>+$6.15M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$31.68M</t>
+          <t>+$30.62M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -916,12 +916,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>+$6.31M</t>
+          <t>+$6.18M</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+$82.82M</t>
+          <t>+$81.04M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -978,12 +978,12 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>+$18.60M</t>
+          <t>+$19.25M</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>+$23.42M</t>
+          <t>+$24.24M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1011,12 +1011,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>+$12.36M</t>
+          <t>+$13.14M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$20.00M</t>
+          <t>+$21.26M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1044,12 +1044,12 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>+$25.25M</t>
+          <t>+$27.33M</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>+$28.16M</t>
+          <t>+$30.47M</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>+$8.12M</t>
+          <t>+$9.19M</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+$9.11M</t>
+          <t>+$10.31M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1176,12 +1176,12 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>+$21.23M</t>
+          <t>+$23.94M</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>+$27.86M</t>
+          <t>+$31.41M</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
@@ -1209,12 +1209,12 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>+$5.23M</t>
+          <t>+$6.07M</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>+$6.13M</t>
+          <t>+$7.12M</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>+$17.51M</t>
+          <t>+$21.01M</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>+$17.55M</t>
+          <t>+$21.06M</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -2480,7 +2480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2530,54 +2530,58 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>4401.35</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="A2" s="6" t="n">
+        <v>4313.32</v>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>392</v>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>+$319.48K</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>+$9.41M</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr"/>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>-$47.39M</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>+$47.41M</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>4403.06</v>
+        <v>4335.33</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>99</v>
+        <v>394</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>-$4.59M</t>
+          <t>-$991.29K</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+$7.30M</t>
+          <t>+$1.11M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -2587,30 +2591,30 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n">
-        <v>4456.36</v>
+        <v>4346.33</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>+$15.29M</t>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>-$73.64M</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>+$18.75M</t>
+          <t>+$74.07M</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -2620,16 +2624,16 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4478.37</v>
+        <v>4368.34</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>407</v>
+        <v>397</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
@@ -2638,144 +2642,132 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>-$3.21M</t>
+          <t>-$6.72M</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>+$5.98M</t>
+          <t>+$6.89M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>4489.37</v>
+        <v>4401.35</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>408</v>
+        <v>400</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>+$7.66M</t>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-$2.75M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$9.33M</t>
+          <t>+$6.89M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>4500.38</v>
+        <v>4403.06</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>409</v>
+        <v>99</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>-$4.59M</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>+$7.30M</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>4456.36</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>405</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>-$1.53M</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>+$3.05M</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>4511.38</v>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>410</v>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>+$53.87M</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>+$58.36M</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>+$9.87M</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>+$19.56M</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>4536.48</v>
+        <v>4511.38</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>102</v>
+        <v>410</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>+$21.91M</t>
+          <t>+$39.68M</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>+$23.76M</t>
+          <t>+$65.18M</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -2791,24 +2783,24 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
-        <v>4566.4</v>
+        <v>4536.48</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>415</v>
+        <v>102</v>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>-$3.74M</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>+$21.91M</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>+$16.81M</t>
+          <t>+$23.76M</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -2818,16 +2810,16 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>4621.41</v>
+        <v>4566.4</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -2836,12 +2828,12 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>-$2.17M</t>
+          <t>-$3.81M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+$22.61M</t>
+          <t>+$16.81M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -2853,10 +2845,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>4676.43</v>
+        <v>4621.41</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -2865,12 +2857,12 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>+$6.37M</t>
+          <t>+$1.54M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$7.70M</t>
+          <t>+$26.29M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -2882,68 +2874,93 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
+        <v>4676.43</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>425</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>+$6.38M</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>+$7.72M</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>4714.38</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B14" s="2" t="n">
         <v>106</v>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>+$7.68M</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>+$7.70M</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
         <v>4731.45</v>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B15" s="2" t="n">
         <v>430</v>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>+$10.43M</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>+$10.45M</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>+$10.41M</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>+$10.42M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G14"/>
+  <autoFilter ref="A1:G15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2955,7 +2972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3291,12 +3308,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+$6.31M</t>
+          <t>+$6.18M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>+$82.82M</t>
+          <t>+$81.04M</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -3309,28 +3326,28 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>7806.15</v>
+        <v>4346.33</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>778</v>
+        <v>395</v>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>+$61.96M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>-$73.64M</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>+$62.03M</t>
+          <t>+$74.07M</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -3340,7 +3357,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3363,12 +3380,12 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>+$53.87M</t>
+          <t>+$39.68M</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>+$58.36M</t>
+          <t>+$65.18M</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -3385,28 +3402,28 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>29585.06</v>
+        <v>7806.15</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>718</v>
+        <v>778</v>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>-$10.78M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>+$61.96M</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>+$46.81M</t>
+          <t>+$62.03M</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -3416,183 +3433,187 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>4313.32</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>392</v>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>-$47.39M</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>+$47.41M</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>29585.06</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>718</v>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>-$10.78M</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>+$46.81M</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
-        <v>7710.04</v>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>7700</v>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>-$11.05M</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>+$45.97M</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="B15" s="2" t="n">
+        <v>7756.05</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>773</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>+$13.66M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+$43.78M</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>3018</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>+$40.40M</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>+$42.85M</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>7756.05</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>773</v>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>+$13.66M</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>+$43.78M</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>3018</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>300</v>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>+$40.40M</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>+$42.85M</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>29256.41</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>710</v>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>+$2.45M</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>+$40.87M</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>2992.85</v>
+        <v>7710.04</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>297.5</v>
+        <v>7700</v>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>+$31.12M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>-$9.92M</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>+$35.07M</t>
+          <t>+$41.28M</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -3602,251 +3623,251 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>29256.41</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>710</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>+$2.45M</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>+$40.87M</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>2992.85</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>297.5</v>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>+$31.12M</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>+$35.07M</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B20" s="6" t="n">
+        <v>7810.04</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>7800</v>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>+$23.94M</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>+$31.41M</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>7750.04</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>7740</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+$6.15M</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>+$30.62M</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
         <v>7735.04</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C22" s="2" t="n">
         <v>7725</v>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>+$70.66K</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>+$33.13M</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+$65.08K</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>+$30.51M</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
-        <v>7750.04</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>7740</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="B23" s="6" t="n">
+        <v>7790.04</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>7780</v>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>+$6.36M</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>+$31.68M</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>7730.04</v>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>7720</v>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>-$7.18M</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>+$28.19M</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>7790.04</v>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>7780</v>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>+$25.25M</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>+$28.16M</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>+$27.33M</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>+$30.47M</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="n">
-        <v>7810.04</v>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>7800</v>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>+$21.23M</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>+$27.86M</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>7826.19</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>780</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>+$25.85M</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>+$25.88M</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>7655.84</v>
+        <v>4621.41</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>763</v>
+        <v>420</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>+$1.70M</t>
+          <t>+$1.54M</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>+$25.61M</t>
+          <t>+$26.29M</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -3859,28 +3880,28 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>2937.52</v>
+        <v>7826.19</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>292</v>
+        <v>780</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-$21.02M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>+$25.85M</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>+$25.53M</t>
+          <t>+$25.88M</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -3893,112 +3914,108 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>29749.38</v>
+        <v>7730.04</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>722</v>
+        <v>7720</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>+$18.35M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>-$6.58M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>+$23.97M</t>
+          <t>+$25.80M</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>7655.84</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>763</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>+$1.70M</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>+$25.61M</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n">
-        <v>4536.48</v>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>102</v>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>+$21.91M</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>+$23.76M</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>29769.92</v>
+        <v>2937.52</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>722.5</v>
+        <v>292</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>+$20.06M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>-$21.02M</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>+$23.69M</t>
+          <t>+$25.53M</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -4019,12 +4036,12 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>+$18.60M</t>
+          <t>+$19.25M</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+$23.42M</t>
+          <t>+$24.24M</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -4041,100 +4058,100 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>7796.13</v>
+        <v>29749.38</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>777</v>
+        <v>722</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>+$23.27M</t>
+          <t>+$18.35M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$23.39M</t>
+          <t>+$23.97M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
-        <v>4621.41</v>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>420</v>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>-$2.17M</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>+$22.61M</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr"/>
+      <c r="B31" s="6" t="n">
+        <v>4536.48</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>102</v>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>+$21.91M</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>+$23.76M</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>7725.04</v>
+        <v>29769.92</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>7715</v>
+        <v>722.5</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>+$4.35M</t>
+          <t>+$20.06M</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>+$21.62M</t>
+          <t>+$23.69M</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -4155,32 +4172,36 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>7625.78</v>
+        <v>7796.13</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>760</v>
+        <v>777</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>-$16.51M</t>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>+$23.27M</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>+$21.19M</t>
+          <t>+$23.39M</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -4201,12 +4222,12 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>+$12.36M</t>
+          <t>+$13.14M</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>+$20.00M</t>
+          <t>+$21.26M</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -4221,42 +4242,38 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="n">
-        <v>4456.36</v>
-      </c>
-      <c r="C35" s="6" t="n">
-        <v>405</v>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>+$15.29M</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>+$18.75M</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>7625.78</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>760</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>-$16.51M</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>+$21.19M</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -4277,12 +4294,12 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>+$17.51M</t>
+          <t>+$21.01M</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>+$17.55M</t>
+          <t>+$21.06M</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -4297,182 +4314,174 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>7725.04</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>7715</v>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>+$3.95M</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>+$19.63M</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>4456.36</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>405</v>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>+$9.87M</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>+$19.56M</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n">
+      <c r="B39" s="6" t="n">
         <v>29872.62</v>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="C39" s="6" t="n">
         <v>725</v>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E39" s="9" t="inlineStr">
         <is>
           <t>+$16.75M</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>+$17.20M</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n">
+      <c r="B40" s="2" t="n">
         <v>4566.4</v>
       </c>
-      <c r="C38" s="6" t="n">
+      <c r="C40" s="2" t="n">
         <v>415</v>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>-$3.74M</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>-$3.81M</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>+$16.81M</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H38" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>29174.25</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>708</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>-$8.24M</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>+$16.51M</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="n">
-        <v>29051.01</v>
-      </c>
-      <c r="C40" s="6" t="n">
-        <v>705</v>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>-$8.46M</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>+$15.76M</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H40" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>2997.88</v>
+        <v>29174.25</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>298</v>
+        <v>708</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>+$6.04M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>-$8.24M</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>+$13.68M</t>
+          <t>+$16.51M</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -4489,112 +4498,112 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="n">
+        <v>29051.01</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>705</v>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>-$8.46M</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>+$15.76M</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>2997.88</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>298</v>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>+$6.04M</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>+$13.68M</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B42" s="6" t="n">
+      <c r="B44" s="6" t="n">
         <v>90.67</v>
       </c>
-      <c r="C42" s="6" t="n">
+      <c r="C44" s="6" t="n">
         <v>140</v>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D44" s="7" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>-$5.74M</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>+$10.87M</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n">
-        <v>4731.45</v>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>430</v>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>+$10.43M</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>+$10.45M</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H43" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n">
-        <v>29708.3</v>
-      </c>
-      <c r="C44" s="2" t="n">
-        <v>721</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>+$6.05M</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>+$10.12M</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="H44" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4603,28 +4612,28 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>7660.04</v>
+        <v>4731.45</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>7650</v>
+        <v>430</v>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>-$4.50M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>+$10.41M</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>+$9.70M</t>
+          <t>+$10.42M</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -4637,188 +4646,188 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>4401.35</v>
+        <v>7805.04</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>400</v>
+        <v>7795</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>+$319.48K</t>
+          <t>+$9.19M</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>+$9.41M</t>
+          <t>+$10.31M</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>29708.3</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>721</v>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>+$6.05M</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>+$10.12M</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="n">
+        <v>28845.61</v>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>700</v>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>-$7.99M</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>+$9.35M</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="n">
+        <v>93.90000000000001</v>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>+$8.52M</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>+$8.68M</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>7660.04</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>7650</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>-$3.94M</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>+$8.49M</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="n">
-        <v>28845.61</v>
-      </c>
-      <c r="C47" s="6" t="n">
-        <v>700</v>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>-$7.99M</t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>+$9.35M</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H47" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>4489.37</v>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>408</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>+$7.66M</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>+$9.33M</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n">
-        <v>7805.04</v>
-      </c>
-      <c r="C49" s="2" t="n">
-        <v>7795</v>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>+$8.12M</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>+$9.11M</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="n">
-        <v>93.90000000000001</v>
-      </c>
-      <c r="C50" s="6" t="n">
-        <v>145</v>
-      </c>
-      <c r="D50" s="7" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E50" s="9" t="inlineStr">
-        <is>
-          <t>+$8.52M</t>
-        </is>
-      </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>+$8.68M</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H50" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -4839,12 +4848,12 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>+$6.37M</t>
+          <t>+$6.38M</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>+$7.70M</t>
+          <t>+$7.72M</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -4929,74 +4938,74 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>30283.43</v>
+        <v>7825.04</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>735</v>
+        <v>7815</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>+$7.06M</t>
+          <t>+$6.07M</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>+$7.06M</t>
+          <t>+$7.12M</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>7825.04</v>
+        <v>30283.43</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>7815</v>
+        <v>735</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>+$5.23M</t>
+          <t>+$7.06M</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>+$6.13M</t>
+          <t>+$7.06M</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -5005,10 +5014,10 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>4478.37</v>
+        <v>4368.34</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>407</v>
+        <v>397</v>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
@@ -5017,62 +5026,54 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>-$3.21M</t>
+          <t>-$6.72M</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>+$5.98M</t>
+          <t>+$6.89M</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>29831.54</v>
+        <v>4401.35</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>724</v>
+        <v>400</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
-        <is>
-          <t>+$4.28M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>-$2.75M</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>+$4.60M</t>
+          <t>+$6.89M</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -5081,24 +5082,24 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>29092.09</v>
+        <v>29831.54</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>706</v>
+        <v>724</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>-$777.38K</t>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>+$4.28M</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>+$4.51M</t>
+          <t>+$4.60M</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -5108,155 +5109,155 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>29092.09</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>706</v>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>-$777.38K</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>+$4.51M</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B59" s="2" t="n">
+      <c r="B60" s="2" t="n">
         <v>92.61</v>
       </c>
-      <c r="C59" s="2" t="n">
+      <c r="C60" s="2" t="n">
         <v>143</v>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>+$3.26M</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>+$4.17M</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="n">
-        <v>29689.18</v>
-      </c>
-      <c r="C60" s="6" t="n">
-        <v>29600</v>
-      </c>
-      <c r="D60" s="7" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>-$3.26M</t>
-        </is>
-      </c>
-      <c r="F60" s="7" t="inlineStr">
-        <is>
-          <t>+$3.97M</t>
-        </is>
-      </c>
-      <c r="G60" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H60" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="n">
+        <v>29689.18</v>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>29600</v>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>-$3.26M</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>+$3.97M</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B61" s="6" t="n">
+      <c r="B62" s="6" t="n">
         <v>89.37</v>
       </c>
-      <c r="C61" s="6" t="n">
+      <c r="C62" s="6" t="n">
         <v>138</v>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E61" s="9" t="inlineStr">
+      <c r="E62" s="9" t="inlineStr">
         <is>
           <t>+$2.67M</t>
         </is>
       </c>
-      <c r="F61" s="7" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>+$3.90M</t>
         </is>
       </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H61" s="7" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="n">
-        <v>4500.38</v>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>409</v>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>-$1.53M</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>+$3.05M</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5411,36 +5412,40 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>29639.18</v>
+        <v>4335.33</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>29550</v>
+        <v>394</v>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>+$9.43K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>-$991.29K</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>+$575.49K</t>
+          <t>+$1.11M</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -5449,10 +5454,10 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>29389.18</v>
+        <v>29639.18</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>29300</v>
+        <v>29550</v>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
@@ -5461,12 +5466,12 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>+$123.83K</t>
+          <t>+$9.43K</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>+$435.16K</t>
+          <t>+$575.49K</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -5483,39 +5488,73 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
+        <v>29389.18</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>29300</v>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>+$123.83K</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>+$435.16K</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
         <v>29619.18</v>
       </c>
-      <c r="C69" s="2" t="n">
+      <c r="C70" s="2" t="n">
         <v>29530</v>
       </c>
-      <c r="D69" s="3" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>-$4.72K</t>
         </is>
       </c>
-      <c r="F69" s="3" t="inlineStr">
+      <c r="F70" s="3" t="inlineStr">
         <is>
           <t>+$221.71K</t>
         </is>
       </c>
-      <c r="G69" s="3" t="inlineStr">
+      <c r="G70" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H69" s="3" t="inlineStr">
+      <c r="H70" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H69"/>
+  <autoFilter ref="A1:H70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>